<commit_message>
fix(docs): changing type data in specific cells
</commit_message>
<xml_diff>
--- a/docs/template_disposisi.xlsx
+++ b/docs/template_disposisi.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Code\Project\api-smartdoku\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annas\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8986410B-EFE4-4FD4-91BD-4270B5B2627F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204A483F-A1C0-455B-B452-E1F56612813B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="330" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="disposisi" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -167,11 +166,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="@\ &quot; :&quot;"/>
     <numFmt numFmtId="165" formatCode="dd\ mmmm\,\ yyyy"/>
+    <numFmt numFmtId="168" formatCode="[$-409]h:mm\ AM/PM;@"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,50 +183,61 @@
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -394,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -442,6 +453,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -499,6 +516,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -514,16 +543,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -535,6 +570,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -549,30 +593,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -585,14 +605,11 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1729,7 +1746,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I26"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
@@ -1742,85 +1759,85 @@
     <col min="9" max="9" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="16" customFormat="1" ht="15.75">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:9" s="16" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="25"/>
-    </row>
-    <row r="2" spans="1:9" s="17" customFormat="1" ht="21">
-      <c r="A2" s="26" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" s="17" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="28"/>
-    </row>
-    <row r="3" spans="1:9" s="17" customFormat="1" ht="21">
-      <c r="A3" s="26" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="30"/>
+    </row>
+    <row r="3" spans="1:9" s="17" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="28"/>
-    </row>
-    <row r="4" spans="1:9" s="2" customFormat="1">
-      <c r="A4" s="29" t="s">
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="30"/>
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="31"/>
-    </row>
-    <row r="5" spans="1:9" s="22" customFormat="1">
-      <c r="A5" s="29" t="s">
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="33"/>
+    </row>
+    <row r="5" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="31"/>
-    </row>
-    <row r="6" spans="1:9" s="2" customFormat="1">
-      <c r="A6" s="29" t="s">
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="33"/>
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="31"/>
-    </row>
-    <row r="7" spans="1:9" s="14" customFormat="1" ht="15.75" customHeight="1">
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="33"/>
+    </row>
+    <row r="7" spans="1:9" s="14" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19"/>
       <c r="B7" s="20"/>
       <c r="C7" s="20"/>
@@ -1831,68 +1848,68 @@
       <c r="H7" s="20"/>
       <c r="I7" s="21"/>
     </row>
-    <row r="8" spans="1:9" s="18" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A8" s="33" t="s">
+    <row r="8" spans="1:9" s="18" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="35"/>
-    </row>
-    <row r="9" spans="1:9" s="18" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A9" s="36"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="38"/>
-    </row>
-    <row r="10" spans="1:9" s="14" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A10" s="60" t="s">
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="37"/>
+    </row>
+    <row r="9" spans="1:9" s="18" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="38"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="40"/>
+    </row>
+    <row r="10" spans="1:9" s="14" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="61"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="72" t="s">
+      <c r="B10" s="54"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="40"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="60" t="s">
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="42"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="61"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="73" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-      <c r="I11" s="53"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="62" t="s">
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="61"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="44"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
       <c r="F12" s="3" t="s">
         <v>3</v>
       </c>
@@ -1902,76 +1919,76 @@
       <c r="H12" s="3"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="33" customHeight="1">
-      <c r="A13" s="64"/>
-      <c r="B13" s="65"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="46"/>
+    <row r="13" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="46"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="51"/>
+      <c r="E13" s="52"/>
       <c r="F13" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="51" t="s">
+      <c r="G13" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="51"/>
+      <c r="H13" s="59"/>
       <c r="I13" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="30.75" customHeight="1">
-      <c r="A14" s="74" t="s">
+    <row r="14" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="64" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="48"/>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="66" t="s">
+      <c r="B14" s="45"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="56"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B15" s="67"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
-      <c r="I15" s="50"/>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="68" t="s">
+      <c r="B15" s="63"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="58"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="69"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="49"/>
-      <c r="I16" s="50"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A17" s="70" t="s">
+      <c r="B16" s="72"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="75"/>
+      <c r="F16" s="75"/>
+      <c r="G16" s="75"/>
+      <c r="H16" s="75"/>
+      <c r="I16" s="76"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B17" s="71"/>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="54"/>
-      <c r="H17" s="54"/>
-      <c r="I17" s="55"/>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="B17" s="74"/>
+      <c r="C17" s="65"/>
+      <c r="D17" s="65"/>
+      <c r="E17" s="65"/>
+      <c r="F17" s="65"/>
+      <c r="G17" s="65"/>
+      <c r="H17" s="65"/>
+      <c r="I17" s="66"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>19</v>
       </c>
@@ -1986,7 +2003,7 @@
       <c r="H18" s="9"/>
       <c r="I18" s="10"/>
     </row>
-    <row r="19" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1">
+    <row r="19" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="12" t="s">
         <v>21</v>
@@ -2003,7 +2020,7 @@
       </c>
       <c r="I19" s="13"/>
     </row>
-    <row r="20" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1">
+    <row r="20" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
       <c r="B20" s="12" t="s">
         <v>24</v>
@@ -2020,7 +2037,7 @@
       </c>
       <c r="I20" s="13"/>
     </row>
-    <row r="21" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1">
+    <row r="21" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="12" t="s">
         <v>27</v>
@@ -2037,7 +2054,7 @@
       </c>
       <c r="I21" s="13"/>
     </row>
-    <row r="22" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1">
+    <row r="22" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
       <c r="B22" s="12" t="s">
         <v>30</v>
@@ -2054,7 +2071,7 @@
       </c>
       <c r="I22" s="13"/>
     </row>
-    <row r="23" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1">
+    <row r="23" spans="1:9" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11"/>
       <c r="B23" s="12" t="s">
         <v>33</v>
@@ -2071,7 +2088,7 @@
       </c>
       <c r="I23" s="13"/>
     </row>
-    <row r="24" spans="1:9" s="1" customFormat="1" ht="25.5" customHeight="1">
+    <row r="24" spans="1:9" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11"/>
       <c r="B24" s="12" t="s">
         <v>36</v>
@@ -2086,33 +2103,33 @@
       <c r="H24" s="12"/>
       <c r="I24" s="13"/>
     </row>
-    <row r="25" spans="1:9" ht="98.25" customHeight="1">
-      <c r="A25" s="56" t="s">
+    <row r="25" spans="1:9" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="56"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="56"/>
-    </row>
-    <row r="26" spans="1:9" s="14" customFormat="1" ht="196.5" customHeight="1">
-      <c r="A26" s="56" t="s">
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
+      <c r="E25" s="67"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="67"/>
+      <c r="I25" s="67"/>
+    </row>
+    <row r="26" spans="1:9" s="14" customFormat="1" ht="196.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="56"/>
-      <c r="C26" s="56"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="56"/>
-      <c r="F26" s="57" t="s">
+      <c r="B26" s="67"/>
+      <c r="C26" s="67"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="67"/>
+      <c r="F26" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="G26" s="58"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="59"/>
+      <c r="G26" s="69"/>
+      <c r="H26" s="69"/>
+      <c r="I26" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>